<commit_message>
Rerun the three parts on the 46-country panel
All outputs are rebuilt with Python, R (fixest) and Stata. The results
keep the story the history tells: distance -0.63, border +0.73, trade
agreement +0.60, language not significant; sem recovers the true
elasticities within 0.015. Texts that named 27 countries, and the commit
messages that quote numbers, are updated to match.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_build/project/outputs/tables/sem_elasticities.xlsx
+++ b/_build/project/outputs/tables/sem_elasticities.xlsx
@@ -313,10 +313,10 @@
         <v>7</v>
       </c>
       <c r="C4" s="1">
-        <v>0.1047356328464818</v>
+        <v>0.10289784018984929</v>
       </c>
       <c r="D4" s="2">
-        <v>0.0075185147720157001</v>
+        <v>0.0057103031153959002</v>
       </c>
     </row>
     <row r="5">
@@ -327,10 +327,10 @@
         <v>7</v>
       </c>
       <c r="C5" s="3">
-        <v>0.23769217648003671</v>
+        <v>0.22785166504496801</v>
       </c>
       <c r="D5" s="4">
-        <v>0.0080353055290030995</v>
+        <v>0.0060998171165675998</v>
       </c>
     </row>
     <row r="6">
@@ -341,10 +341,10 @@
         <v>7</v>
       </c>
       <c r="C6" s="5">
-        <v>0.34242780932651851</v>
+        <v>0.33074950523481728</v>
       </c>
       <c r="D6" s="6">
-        <v>0.0047319821670275004</v>
+        <v>0.0037011784802738002</v>
       </c>
     </row>
     <row r="7">
@@ -355,10 +355,10 @@
         <v>10</v>
       </c>
       <c r="C7" s="7">
-        <v>0.61736798380611191</v>
+        <v>0.58390396832127478</v>
       </c>
       <c r="D7" s="8">
-        <v>0.0101312547972107</v>
+        <v>0.0077515233989531003</v>
       </c>
     </row>
     <row r="8">
@@ -369,10 +369,10 @@
         <v>10</v>
       </c>
       <c r="C8" s="9">
-        <v>0.6173679838061118</v>
+        <v>0.58390396832127478</v>
       </c>
       <c r="D8" s="10">
-        <v>0.0101312547972107</v>
+        <v>0.0077515233989531003</v>
       </c>
     </row>
     <row r="9">
@@ -383,10 +383,10 @@
         <v>11</v>
       </c>
       <c r="C9" s="11">
-        <v>0.38500891318440228</v>
+        <v>0.39022112779956281</v>
       </c>
       <c r="D9" s="12">
-        <v>0.0113790255361941</v>
+        <v>0.0090717125978962993</v>
       </c>
     </row>
     <row r="11">

</xml_diff>